<commit_message>
actualizacion de notas de diciembre
</commit_message>
<xml_diff>
--- a/inasistencias-6A-InstrumentalYsistElect/Alumnos-6A-InstrumentalYsistElect.xlsx
+++ b/inasistencias-6A-InstrumentalYsistElect/Alumnos-6A-InstrumentalYsistElect.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="asistencia" sheetId="1" state="visible" r:id="rId3"/>
@@ -1092,7 +1092,7 @@
       <family val="0"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1103,6 +1103,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF4000"/>
+        <bgColor rgb="FFCC0000"/>
       </patternFill>
     </fill>
     <fill>
@@ -1190,6 +1196,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1203,6 +1213,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1222,19 +1236,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1242,11 +1248,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1341,7 +1347,6 @@
           <bgColor rgb="FFCCFFCC"/>
         </patternFill>
       </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </dxf>
     <dxf>
       <font>
@@ -1356,7 +1361,6 @@
           <bgColor rgb="FFFFCCCC"/>
         </patternFill>
       </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </dxf>
     <dxf>
       <font>
@@ -1372,7 +1376,6 @@
           <bgColor rgb="FFCC0000"/>
         </patternFill>
       </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </dxf>
     <dxf>
       <font>
@@ -1436,7 +1439,7 @@
       <rgbColor rgb="FF8BC34A"/>
       <rgbColor rgb="FFFFC107"/>
       <rgbColor rgb="FFFF9800"/>
-      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FFFF4000"/>
       <rgbColor rgb="FF666699"/>
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
@@ -1563,7 +1566,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AM29"/>
+  <dimension ref="A1:AO29"/>
   <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.5"/>
@@ -1719,6 +1722,12 @@
       <c r="AM2" s="3" t="s">
         <v>13</v>
       </c>
+      <c r="AN2" s="6" t="n">
+        <v>45965</v>
+      </c>
+      <c r="AO2" s="6" t="n">
+        <v>45972</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
@@ -1775,11 +1784,11 @@
         <f aca="false">COUNTIF(E3:P3,"T")</f>
         <v>0</v>
       </c>
-      <c r="T3" s="6" t="n">
+      <c r="T3" s="7" t="n">
         <f aca="false">ROUND(Q3+R3/3+S3/4,0)</f>
         <v>8</v>
       </c>
-      <c r="U3" s="7" t="n">
+      <c r="U3" s="8" t="n">
         <f aca="false">ROUND(T3*10/$W$1,0)</f>
         <v>9</v>
       </c>
@@ -1834,7 +1843,7 @@
         <f aca="false">COUNTIF(V3:AG3,"T")</f>
         <v>0</v>
       </c>
-      <c r="AM3" s="8" t="n">
+      <c r="AM3" s="9" t="n">
         <f aca="false">ROUND(AJ3+AK3/2+AL3/4,0)</f>
         <v>8</v>
       </c>
@@ -1894,11 +1903,11 @@
         <f aca="false">COUNTIF(E4:P4,"T")</f>
         <v>0</v>
       </c>
-      <c r="T4" s="6" t="n">
+      <c r="T4" s="7" t="n">
         <f aca="false">ROUND(Q4+R4/3+S4/4,0)</f>
         <v>9</v>
       </c>
-      <c r="U4" s="7" t="n">
+      <c r="U4" s="8" t="n">
         <f aca="false">ROUND(T4*10/$W$1,0)</f>
         <v>10</v>
       </c>
@@ -1953,7 +1962,7 @@
         <f aca="false">COUNTIF(V4:AG4,"T")</f>
         <v>0</v>
       </c>
-      <c r="AM4" s="8" t="n">
+      <c r="AM4" s="9" t="n">
         <f aca="false">ROUND(AJ4+AK4/2+AL4/4,0)</f>
         <v>6</v>
       </c>
@@ -2010,11 +2019,11 @@
         <f aca="false">COUNTIF(E5:P5,"T")</f>
         <v>0</v>
       </c>
-      <c r="T5" s="6" t="n">
+      <c r="T5" s="7" t="n">
         <f aca="false">ROUND(Q5+R5/3+S5/4,0)</f>
         <v>7</v>
       </c>
-      <c r="U5" s="7" t="n">
+      <c r="U5" s="8" t="n">
         <f aca="false">ROUND(T5*10/$W$1,0)</f>
         <v>8</v>
       </c>
@@ -2069,7 +2078,7 @@
         <f aca="false">COUNTIF(V5:AG5,"T")</f>
         <v>0</v>
       </c>
-      <c r="AM5" s="8" t="n">
+      <c r="AM5" s="9" t="n">
         <f aca="false">ROUND(AJ5+AK5/2+AL5/4,0)</f>
         <v>8</v>
       </c>
@@ -2126,11 +2135,11 @@
         <f aca="false">COUNTIF(E6:P6,"T")</f>
         <v>0</v>
       </c>
-      <c r="T6" s="6" t="n">
+      <c r="T6" s="7" t="n">
         <f aca="false">ROUND(Q6+R6/3+S6/4,0)</f>
         <v>7</v>
       </c>
-      <c r="U6" s="7" t="n">
+      <c r="U6" s="8" t="n">
         <f aca="false">ROUND(T6*10/$W$1,0)</f>
         <v>8</v>
       </c>
@@ -2185,7 +2194,7 @@
         <f aca="false">COUNTIF(V6:AG6,"T")</f>
         <v>0</v>
       </c>
-      <c r="AM6" s="8" t="n">
+      <c r="AM6" s="9" t="n">
         <f aca="false">ROUND(AJ6+AK6/2+AL6/4,0)</f>
         <v>10</v>
       </c>
@@ -2194,13 +2203,13 @@
       <c r="A7" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="10" t="s">
         <v>33</v>
       </c>
       <c r="E7" s="2" t="s">
@@ -2245,11 +2254,11 @@
         <f aca="false">COUNTIF(E7:P7,"T")</f>
         <v>0</v>
       </c>
-      <c r="T7" s="10" t="n">
+      <c r="T7" s="12" t="n">
         <f aca="false">ROUND(Q7+R7/3+S7/4,0)</f>
         <v>1</v>
       </c>
-      <c r="U7" s="11" t="n">
+      <c r="U7" s="13" t="n">
         <f aca="false">ROUND(T7*10/$W$1,0)</f>
         <v>1</v>
       </c>
@@ -2271,7 +2280,7 @@
       <c r="AC7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="AD7" s="9" t="s">
+      <c r="AD7" s="10" t="s">
         <v>19</v>
       </c>
       <c r="AE7" s="2" t="s">
@@ -2283,10 +2292,10 @@
       <c r="AG7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="AH7" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="AI7" s="9" t="s">
+      <c r="AH7" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="AI7" s="10" t="s">
         <v>17</v>
       </c>
       <c r="AJ7" s="3" t="n">
@@ -2301,7 +2310,7 @@
         <f aca="false">COUNTIF(V7:AG7,"T")</f>
         <v>0</v>
       </c>
-      <c r="AM7" s="8" t="n">
+      <c r="AM7" s="9" t="n">
         <f aca="false">ROUND(AJ7+AK7/2+AL7/4,0)</f>
         <v>2</v>
       </c>
@@ -2310,13 +2319,13 @@
       <c r="A8" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="10" t="s">
         <v>36</v>
       </c>
       <c r="E8" s="2" t="s">
@@ -2361,11 +2370,11 @@
         <f aca="false">COUNTIF(E8:P8,"T")</f>
         <v>0</v>
       </c>
-      <c r="T8" s="10" t="n">
+      <c r="T8" s="12" t="n">
         <f aca="false">ROUND(Q8+R8/3+S8/4,0)</f>
         <v>0</v>
       </c>
-      <c r="U8" s="11" t="n">
+      <c r="U8" s="13" t="n">
         <f aca="false">ROUND(T8*10/$W$1,0)</f>
         <v>0</v>
       </c>
@@ -2399,10 +2408,10 @@
       <c r="AG8" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="AH8" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="AI8" s="9" t="s">
+      <c r="AH8" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="AI8" s="10" t="s">
         <v>19</v>
       </c>
       <c r="AJ8" s="3" t="n">
@@ -2417,7 +2426,7 @@
         <f aca="false">COUNTIF(V8:AG8,"T")</f>
         <v>0</v>
       </c>
-      <c r="AM8" s="8" t="n">
+      <c r="AM8" s="9" t="n">
         <f aca="false">ROUND(AJ8+AK8/2+AL8/4,0)</f>
         <v>1</v>
       </c>
@@ -2477,11 +2486,11 @@
         <f aca="false">COUNTIF(E9:P9,"T")</f>
         <v>0</v>
       </c>
-      <c r="T9" s="6" t="n">
+      <c r="T9" s="7" t="n">
         <f aca="false">ROUND(Q9+R9/3+S9/4,0)</f>
         <v>9</v>
       </c>
-      <c r="U9" s="7" t="n">
+      <c r="U9" s="8" t="n">
         <f aca="false">ROUND(T9*10/$W$1,0)</f>
         <v>10</v>
       </c>
@@ -2536,7 +2545,7 @@
         <f aca="false">COUNTIF(V9:AG9,"T")</f>
         <v>0</v>
       </c>
-      <c r="AM9" s="8" t="n">
+      <c r="AM9" s="9" t="n">
         <f aca="false">ROUND(AJ9+AK9/2+AL9/4,0)</f>
         <v>10</v>
       </c>
@@ -2596,11 +2605,11 @@
         <f aca="false">COUNTIF(E10:P10,"T")</f>
         <v>0</v>
       </c>
-      <c r="T10" s="6" t="n">
+      <c r="T10" s="7" t="n">
         <f aca="false">ROUND(Q10+R10/3+S10/4,0)</f>
         <v>9</v>
       </c>
-      <c r="U10" s="7" t="n">
+      <c r="U10" s="8" t="n">
         <f aca="false">ROUND(T10*10/$W$1,0)</f>
         <v>10</v>
       </c>
@@ -2655,7 +2664,7 @@
         <f aca="false">COUNTIF(V10:AG10,"T")</f>
         <v>0</v>
       </c>
-      <c r="AM10" s="8" t="n">
+      <c r="AM10" s="9" t="n">
         <f aca="false">ROUND(AJ10+AK10/2+AL10/4,0)</f>
         <v>10</v>
       </c>
@@ -2712,11 +2721,11 @@
         <f aca="false">COUNTIF(E11:P11,"T")</f>
         <v>0</v>
       </c>
-      <c r="T11" s="6" t="n">
+      <c r="T11" s="7" t="n">
         <f aca="false">ROUND(Q11+R11/3+S11/4,0)</f>
         <v>9</v>
       </c>
-      <c r="U11" s="7" t="n">
+      <c r="U11" s="8" t="n">
         <f aca="false">ROUND(T11*10/$W$1,0)</f>
         <v>10</v>
       </c>
@@ -2771,7 +2780,7 @@
         <f aca="false">COUNTIF(V11:AG11,"T")</f>
         <v>0</v>
       </c>
-      <c r="AM11" s="8" t="n">
+      <c r="AM11" s="9" t="n">
         <f aca="false">ROUND(AJ11+AK11/2+AL11/4,0)</f>
         <v>10</v>
       </c>
@@ -2828,11 +2837,11 @@
         <f aca="false">COUNTIF(E12:P12,"T")</f>
         <v>0</v>
       </c>
-      <c r="T12" s="6" t="n">
+      <c r="T12" s="7" t="n">
         <f aca="false">ROUND(Q12+R12/3+S12/4,0)</f>
         <v>8</v>
       </c>
-      <c r="U12" s="7" t="n">
+      <c r="U12" s="8" t="n">
         <f aca="false">ROUND(T12*10/$W$1,0)</f>
         <v>9</v>
       </c>
@@ -2857,7 +2866,7 @@
       <c r="AC12" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="AD12" s="9" t="s">
+      <c r="AD12" s="10" t="s">
         <v>17</v>
       </c>
       <c r="AE12" s="3" t="s">
@@ -2887,7 +2896,7 @@
         <f aca="false">COUNTIF(V12:AG12,"T")</f>
         <v>0</v>
       </c>
-      <c r="AM12" s="8" t="n">
+      <c r="AM12" s="9" t="n">
         <f aca="false">ROUND(AJ12+AK12/2+AL12/4,0)</f>
         <v>8</v>
       </c>
@@ -2944,11 +2953,11 @@
         <f aca="false">COUNTIF(E13:P13,"T")</f>
         <v>0</v>
       </c>
-      <c r="T13" s="6" t="n">
+      <c r="T13" s="7" t="n">
         <f aca="false">ROUND(Q13+R13/3+S13/4,0)</f>
         <v>9</v>
       </c>
-      <c r="U13" s="7" t="n">
+      <c r="U13" s="8" t="n">
         <f aca="false">ROUND(T13*10/$W$1,0)</f>
         <v>10</v>
       </c>
@@ -3003,7 +3012,7 @@
         <f aca="false">COUNTIF(V13:AG13,"T")</f>
         <v>0</v>
       </c>
-      <c r="AM13" s="8" t="n">
+      <c r="AM13" s="9" t="n">
         <f aca="false">ROUND(AJ13+AK13/2+AL13/4,0)</f>
         <v>9</v>
       </c>
@@ -3060,11 +3069,11 @@
         <f aca="false">COUNTIF(E14:P14,"T")</f>
         <v>0</v>
       </c>
-      <c r="T14" s="6" t="n">
+      <c r="T14" s="7" t="n">
         <f aca="false">ROUND(Q14+R14/3+S14/4,0)</f>
         <v>7</v>
       </c>
-      <c r="U14" s="7" t="n">
+      <c r="U14" s="8" t="n">
         <f aca="false">ROUND(T14*10/$W$1,0)</f>
         <v>8</v>
       </c>
@@ -3119,7 +3128,7 @@
         <f aca="false">COUNTIF(V14:AG14,"T")</f>
         <v>0</v>
       </c>
-      <c r="AM14" s="8" t="n">
+      <c r="AM14" s="9" t="n">
         <f aca="false">ROUND(AJ14+AK14/2+AL14/4,0)</f>
         <v>9</v>
       </c>
@@ -3176,11 +3185,11 @@
         <f aca="false">COUNTIF(E15:P15,"T")</f>
         <v>0</v>
       </c>
-      <c r="T15" s="6" t="n">
+      <c r="T15" s="7" t="n">
         <f aca="false">ROUND(Q15+R15/3+S15/4,0)</f>
         <v>6</v>
       </c>
-      <c r="U15" s="7" t="n">
+      <c r="U15" s="8" t="n">
         <f aca="false">ROUND(T15*10/$W$1,0)</f>
         <v>7</v>
       </c>
@@ -3235,7 +3244,7 @@
         <f aca="false">COUNTIF(V15:AG15,"T")</f>
         <v>0</v>
       </c>
-      <c r="AM15" s="8" t="n">
+      <c r="AM15" s="9" t="n">
         <f aca="false">ROUND(AJ15+AK15/2+AL15/4,0)</f>
         <v>9</v>
       </c>
@@ -3292,11 +3301,11 @@
         <f aca="false">COUNTIF(E16:P16,"T")</f>
         <v>0</v>
       </c>
-      <c r="T16" s="6" t="n">
+      <c r="T16" s="7" t="n">
         <f aca="false">ROUND(Q16+R16/3+S16/4,0)</f>
         <v>7</v>
       </c>
-      <c r="U16" s="7" t="n">
+      <c r="U16" s="8" t="n">
         <f aca="false">ROUND(T16*10/$W$1,0)</f>
         <v>8</v>
       </c>
@@ -3351,7 +3360,7 @@
         <f aca="false">COUNTIF(V16:AG16,"T")</f>
         <v>0</v>
       </c>
-      <c r="AM16" s="8" t="n">
+      <c r="AM16" s="9" t="n">
         <f aca="false">ROUND(AJ16+AK16/2+AL16/4,0)</f>
         <v>8</v>
       </c>
@@ -3360,13 +3369,13 @@
       <c r="A17" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="D17" s="9" t="s">
+      <c r="D17" s="10" t="s">
         <v>65</v>
       </c>
       <c r="E17" s="2" t="s">
@@ -3393,7 +3402,7 @@
       <c r="M17" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="N17" s="12" t="n">
+      <c r="N17" s="14" t="n">
         <v>0.548611111111111</v>
       </c>
       <c r="O17" s="2" t="s">
@@ -3414,11 +3423,11 @@
         <f aca="false">COUNTIF(E17:P17,"T")</f>
         <v>0</v>
       </c>
-      <c r="T17" s="10" t="n">
+      <c r="T17" s="12" t="n">
         <f aca="false">ROUND(Q17+R17/3+S17/4,0)</f>
         <v>2</v>
       </c>
-      <c r="U17" s="11" t="n">
+      <c r="U17" s="13" t="n">
         <f aca="false">ROUND(T17*10/$W$1,0)</f>
         <v>2</v>
       </c>
@@ -3452,10 +3461,10 @@
       <c r="AG17" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="AH17" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="AI17" s="9" t="s">
+      <c r="AH17" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="AI17" s="10" t="s">
         <v>19</v>
       </c>
       <c r="AJ17" s="3" t="n">
@@ -3470,7 +3479,7 @@
         <f aca="false">COUNTIF(V17:AG17,"T")</f>
         <v>0</v>
       </c>
-      <c r="AM17" s="8" t="n">
+      <c r="AM17" s="9" t="n">
         <f aca="false">ROUND(AJ17+AK17/2+AL17/4,0)</f>
         <v>1</v>
       </c>
@@ -3479,13 +3488,13 @@
       <c r="A18" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="B18" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C18" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="D18" s="9" t="s">
+      <c r="D18" s="10" t="s">
         <v>69</v>
       </c>
       <c r="E18" s="2" t="s">
@@ -3512,7 +3521,7 @@
       <c r="M18" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="N18" s="12" t="n">
+      <c r="N18" s="14" t="n">
         <v>0.555555555555556</v>
       </c>
       <c r="O18" s="2" t="s">
@@ -3533,11 +3542,11 @@
         <f aca="false">COUNTIF(E18:P18,"T")</f>
         <v>0</v>
       </c>
-      <c r="T18" s="10" t="n">
+      <c r="T18" s="12" t="n">
         <f aca="false">ROUND(Q18+R18/3+S18/4,0)</f>
         <v>2</v>
       </c>
-      <c r="U18" s="11" t="n">
+      <c r="U18" s="13" t="n">
         <f aca="false">ROUND(T18*10/$W$1,0)</f>
         <v>2</v>
       </c>
@@ -3571,10 +3580,10 @@
       <c r="AG18" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="AH18" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="AI18" s="9" t="s">
+      <c r="AH18" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="AI18" s="10" t="s">
         <v>17</v>
       </c>
       <c r="AJ18" s="3" t="n">
@@ -3589,7 +3598,7 @@
         <f aca="false">COUNTIF(V18:AG18,"T")</f>
         <v>0</v>
       </c>
-      <c r="AM18" s="8" t="n">
+      <c r="AM18" s="9" t="n">
         <f aca="false">ROUND(AJ18+AK18/2+AL18/4,0)</f>
         <v>3</v>
       </c>
@@ -3646,11 +3655,11 @@
         <f aca="false">COUNTIF(E19:P19,"T")</f>
         <v>0</v>
       </c>
-      <c r="T19" s="6" t="n">
+      <c r="T19" s="7" t="n">
         <f aca="false">ROUND(Q19+R19/3+S19/4,0)</f>
         <v>8</v>
       </c>
-      <c r="U19" s="7" t="n">
+      <c r="U19" s="8" t="n">
         <f aca="false">ROUND(T19*10/$W$1,0)</f>
         <v>9</v>
       </c>
@@ -3705,7 +3714,7 @@
         <f aca="false">COUNTIF(V19:AG19,"T")</f>
         <v>0</v>
       </c>
-      <c r="AM19" s="8" t="n">
+      <c r="AM19" s="9" t="n">
         <f aca="false">ROUND(AJ19+AK19/2+AL19/4,0)</f>
         <v>9</v>
       </c>
@@ -3744,7 +3753,7 @@
       <c r="M20" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="N20" s="13" t="n">
+      <c r="N20" s="15" t="n">
         <v>0.548611111111111</v>
       </c>
       <c r="O20" s="1" t="s">
@@ -3765,11 +3774,11 @@
         <f aca="false">COUNTIF(E20:P20,"T")</f>
         <v>0</v>
       </c>
-      <c r="T20" s="6" t="n">
+      <c r="T20" s="7" t="n">
         <f aca="false">ROUND(Q20+R20/3+S20/4,0)</f>
         <v>8</v>
       </c>
-      <c r="U20" s="7" t="n">
+      <c r="U20" s="8" t="n">
         <f aca="false">ROUND(T20*10/$W$1,0)</f>
         <v>9</v>
       </c>
@@ -3824,7 +3833,7 @@
         <f aca="false">COUNTIF(V20:AG20,"T")</f>
         <v>0</v>
       </c>
-      <c r="AM20" s="8" t="n">
+      <c r="AM20" s="9" t="n">
         <f aca="false">ROUND(AJ20+AK20/2+AL20/4,0)</f>
         <v>9</v>
       </c>
@@ -3881,11 +3890,11 @@
         <f aca="false">COUNTIF(E21:P21,"T")</f>
         <v>0</v>
       </c>
-      <c r="T21" s="6" t="n">
+      <c r="T21" s="7" t="n">
         <f aca="false">ROUND(Q21+R21/3+S21/4,0)</f>
         <v>9</v>
       </c>
-      <c r="U21" s="7" t="n">
+      <c r="U21" s="8" t="n">
         <f aca="false">ROUND(T21*10/$W$1,0)</f>
         <v>10</v>
       </c>
@@ -3940,7 +3949,7 @@
         <f aca="false">COUNTIF(V21:AG21,"T")</f>
         <v>0</v>
       </c>
-      <c r="AM21" s="8" t="n">
+      <c r="AM21" s="9" t="n">
         <f aca="false">ROUND(AJ21+AK21/2+AL21/4,0)</f>
         <v>6</v>
       </c>
@@ -3979,7 +3988,7 @@
       <c r="M22" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="N22" s="13" t="n">
+      <c r="N22" s="15" t="n">
         <v>0.576388888888889</v>
       </c>
       <c r="O22" s="1" t="s">
@@ -4000,11 +4009,11 @@
         <f aca="false">COUNTIF(E22:P22,"T")</f>
         <v>1</v>
       </c>
-      <c r="T22" s="6" t="n">
+      <c r="T22" s="7" t="n">
         <f aca="false">ROUND(Q22+R22/3+S22/4,0)</f>
         <v>1</v>
       </c>
-      <c r="U22" s="7" t="n">
+      <c r="U22" s="8" t="n">
         <f aca="false">ROUND(T22*10/$W$1,0)</f>
         <v>1</v>
       </c>
@@ -4056,7 +4065,7 @@
         <f aca="false">COUNTIF(V22:AG22,"T")</f>
         <v>0</v>
       </c>
-      <c r="AM22" s="8" t="n">
+      <c r="AM22" s="9" t="n">
         <f aca="false">ROUND(AJ22+AK22/2+AL22/4,0)</f>
         <v>1</v>
       </c>
@@ -4113,11 +4122,11 @@
         <f aca="false">COUNTIF(E23:P23,"T")</f>
         <v>0</v>
       </c>
-      <c r="T23" s="6" t="n">
+      <c r="T23" s="7" t="n">
         <f aca="false">ROUND(Q23+R23/3+S23/4,0)</f>
         <v>9</v>
       </c>
-      <c r="U23" s="7" t="n">
+      <c r="U23" s="8" t="n">
         <f aca="false">ROUND(T23*10/$W$1,0)</f>
         <v>10</v>
       </c>
@@ -4172,7 +4181,7 @@
         <f aca="false">COUNTIF(V23:AG23,"T")</f>
         <v>0</v>
       </c>
-      <c r="AM23" s="8" t="n">
+      <c r="AM23" s="9" t="n">
         <f aca="false">ROUND(AJ23+AK23/2+AL23/4,0)</f>
         <v>10</v>
       </c>
@@ -4229,11 +4238,11 @@
         <f aca="false">COUNTIF(E24:P24,"T")</f>
         <v>0</v>
       </c>
-      <c r="T24" s="6" t="n">
+      <c r="T24" s="7" t="n">
         <f aca="false">ROUND(Q24+R24/3+S24/4,0)</f>
         <v>7</v>
       </c>
-      <c r="U24" s="7" t="n">
+      <c r="U24" s="8" t="n">
         <f aca="false">ROUND(T24*10/$W$1,0)</f>
         <v>8</v>
       </c>
@@ -4288,7 +4297,7 @@
         <f aca="false">COUNTIF(V24:AG24,"T")</f>
         <v>0</v>
       </c>
-      <c r="AM24" s="8" t="n">
+      <c r="AM24" s="9" t="n">
         <f aca="false">ROUND(AJ24+AK24/2+AL24/4,0)</f>
         <v>9</v>
       </c>
@@ -4345,11 +4354,11 @@
         <f aca="false">COUNTIF(E25:P25,"T")</f>
         <v>0</v>
       </c>
-      <c r="T25" s="6" t="n">
+      <c r="T25" s="7" t="n">
         <f aca="false">ROUND(Q25+R25/3+S25/4,0)</f>
         <v>8</v>
       </c>
-      <c r="U25" s="7" t="n">
+      <c r="U25" s="8" t="n">
         <f aca="false">ROUND(T25*10/$W$1,0)</f>
         <v>9</v>
       </c>
@@ -4404,7 +4413,7 @@
         <f aca="false">COUNTIF(V25:AG25,"T")</f>
         <v>0</v>
       </c>
-      <c r="AM25" s="8" t="n">
+      <c r="AM25" s="9" t="n">
         <f aca="false">ROUND(AJ25+AK25/2+AL25/4,0)</f>
         <v>10</v>
       </c>
@@ -4461,11 +4470,11 @@
         <f aca="false">COUNTIF(E26:P26,"T")</f>
         <v>0</v>
       </c>
-      <c r="T26" s="6" t="n">
+      <c r="T26" s="7" t="n">
         <f aca="false">ROUND(Q26+R26/3+S26/4,0)</f>
         <v>8</v>
       </c>
-      <c r="U26" s="7" t="n">
+      <c r="U26" s="8" t="n">
         <f aca="false">ROUND(T26*10/$W$1,0)</f>
         <v>9</v>
       </c>
@@ -4499,7 +4508,7 @@
       <c r="AF26" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="AG26" s="9" t="s">
+      <c r="AG26" s="10" t="s">
         <v>17</v>
       </c>
       <c r="AH26" s="2" t="s">
@@ -4520,7 +4529,7 @@
         <f aca="false">COUNTIF(V26:AG26,"T")</f>
         <v>0</v>
       </c>
-      <c r="AM26" s="8" t="n">
+      <c r="AM26" s="9" t="n">
         <f aca="false">ROUND(AJ26+AK26/2+AL26/4,0)</f>
         <v>10</v>
       </c>
@@ -4577,11 +4586,11 @@
         <f aca="false">COUNTIF(E27:P27,"T")</f>
         <v>0</v>
       </c>
-      <c r="T27" s="6" t="n">
+      <c r="T27" s="7" t="n">
         <f aca="false">ROUND(Q27+R27/3+S27/4,0)</f>
         <v>9</v>
       </c>
-      <c r="U27" s="7" t="n">
+      <c r="U27" s="8" t="n">
         <f aca="false">ROUND(T27*10/$W$1,0)</f>
         <v>10</v>
       </c>
@@ -4636,7 +4645,7 @@
         <f aca="false">COUNTIF(V27:AG27,"T")</f>
         <v>0</v>
       </c>
-      <c r="AM27" s="8" t="n">
+      <c r="AM27" s="9" t="n">
         <f aca="false">ROUND(AJ27+AK27/2+AL27/4,0)</f>
         <v>9</v>
       </c>
@@ -4645,13 +4654,13 @@
       <c r="A28" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="B28" s="9" t="s">
+      <c r="B28" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="C28" s="9" t="s">
+      <c r="C28" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="D28" s="9" t="s">
+      <c r="D28" s="10" t="s">
         <v>100</v>
       </c>
       <c r="E28" s="2" t="s">
@@ -4678,7 +4687,7 @@
       <c r="M28" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="N28" s="12" t="n">
+      <c r="N28" s="14" t="n">
         <v>0.548611111111111</v>
       </c>
       <c r="O28" s="2" t="s">
@@ -4699,11 +4708,11 @@
         <f aca="false">COUNTIF(E28:P28,"T")</f>
         <v>0</v>
       </c>
-      <c r="T28" s="10" t="n">
+      <c r="T28" s="12" t="n">
         <f aca="false">ROUND(Q28+R28/3+S28/4,0)</f>
         <v>0</v>
       </c>
-      <c r="U28" s="11" t="n">
+      <c r="U28" s="13" t="n">
         <f aca="false">ROUND(T28*10/$W$1,0)</f>
         <v>0</v>
       </c>
@@ -4740,10 +4749,10 @@
       <c r="AG28" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="AH28" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="AI28" s="9" t="s">
+      <c r="AH28" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="AI28" s="10" t="s">
         <v>19</v>
       </c>
       <c r="AJ28" s="3" t="n">
@@ -4758,7 +4767,7 @@
         <f aca="false">COUNTIF(V28:AG28,"T")</f>
         <v>0</v>
       </c>
-      <c r="AM28" s="8" t="n">
+      <c r="AM28" s="9" t="n">
         <f aca="false">ROUND(AJ28+AK28/2+AL28/4,0)</f>
         <v>1</v>
       </c>
@@ -4833,11 +4842,11 @@
         <f aca="false">COUNTIF(AG3:AG28,"p")</f>
         <v>15</v>
       </c>
-      <c r="AH29" s="9" t="n">
+      <c r="AH29" s="10" t="n">
         <f aca="false">COUNTIF(AH3:AH28,"p")</f>
         <v>13</v>
       </c>
-      <c r="AI29" s="9"/>
+      <c r="AI29" s="10"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="AM3:AM28">
@@ -5715,10 +5724,10 @@
       <c r="Y1" s="4"/>
       <c r="Z1" s="1"/>
       <c r="AA1" s="1"/>
-      <c r="AD1" s="0" t="s">
+      <c r="AD1" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="AF1" s="0" t="s">
+      <c r="AF1" s="1" t="s">
         <v>104</v>
       </c>
     </row>
@@ -5801,22 +5810,22 @@
       <c r="AA2" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="AB2" s="0" t="s">
+      <c r="AB2" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="AC2" s="0" t="s">
+      <c r="AC2" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="AD2" s="0" t="s">
+      <c r="AD2" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="AE2" s="0" t="s">
+      <c r="AE2" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="AF2" s="0" t="s">
+      <c r="AF2" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="AG2" s="0" t="s">
+      <c r="AG2" s="1" t="s">
         <v>125</v>
       </c>
     </row>
@@ -5847,14 +5856,14 @@
         <f aca="false">ROUND(AVERAGE(C3,E3,J3),0)</f>
         <v>8</v>
       </c>
-      <c r="L3" s="8" t="str">
+      <c r="L3" s="9" t="str">
         <f aca="false">IF(K3&lt;7,"TEP","TEA")</f>
         <v>TEA</v>
       </c>
       <c r="M3" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="O3" s="7" t="n">
+      <c r="O3" s="8" t="n">
         <v>9</v>
       </c>
       <c r="P3" s="1" t="n">
@@ -5867,38 +5876,38 @@
       <c r="R3" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="S3" s="8" t="n">
+      <c r="S3" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(P3:R3),0)</f>
         <v>8</v>
       </c>
-      <c r="T3" s="8"/>
-      <c r="U3" s="8"/>
-      <c r="V3" s="8"/>
+      <c r="T3" s="9"/>
+      <c r="U3" s="9"/>
+      <c r="V3" s="9"/>
       <c r="Y3" s="1" t="n">
         <v>8</v>
       </c>
       <c r="Z3" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="AA3" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC3" s="0" t="n">
+      <c r="AA3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC3" s="1" t="n">
         <f aca="false">AA3+AB3/2</f>
         <v>1</v>
       </c>
-      <c r="AD3" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="AE3" s="15" t="n">
+      <c r="AD3" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="AE3" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(Y3,Z3,AC3),0)</f>
         <v>5</v>
       </c>
-      <c r="AF3" s="15" t="n">
+      <c r="AF3" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(AD3,AE3),0)</f>
         <v>7</v>
       </c>
-      <c r="AG3" s="15" t="n">
+      <c r="AG3" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(S3,AF3),0)</f>
         <v>8</v>
       </c>
@@ -5939,14 +5948,14 @@
         <f aca="false">ROUND(AVERAGE(C4,E4,J4),0)</f>
         <v>4</v>
       </c>
-      <c r="L4" s="8" t="str">
+      <c r="L4" s="9" t="str">
         <f aca="false">IF(K4&lt;7,"TEP","TEA")</f>
         <v>TEP</v>
       </c>
       <c r="M4" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="O4" s="7" t="n">
+      <c r="O4" s="8" t="n">
         <v>10</v>
       </c>
       <c r="P4" s="1" t="n">
@@ -5959,13 +5968,13 @@
       <c r="R4" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="S4" s="8" t="n">
+      <c r="S4" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(P4:R4),0)</f>
         <v>7</v>
       </c>
-      <c r="T4" s="8"/>
-      <c r="U4" s="8"/>
-      <c r="V4" s="8"/>
+      <c r="T4" s="9"/>
+      <c r="U4" s="9"/>
+      <c r="V4" s="9"/>
       <c r="W4" s="1" t="n">
         <v>7</v>
       </c>
@@ -5975,25 +5984,25 @@
       <c r="Z4" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="AA4" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC4" s="15" t="n">
+      <c r="AA4" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC4" s="1" t="n">
         <f aca="false">AA4+AB4/2</f>
         <v>10</v>
       </c>
-      <c r="AD4" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="AE4" s="15" t="n">
+      <c r="AD4" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="AE4" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(Y4,Z4,AC4),0)</f>
         <v>8</v>
       </c>
-      <c r="AF4" s="15" t="n">
+      <c r="AF4" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(AD4,AE4),0)</f>
         <v>9</v>
       </c>
-      <c r="AG4" s="15" t="n">
+      <c r="AG4" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(S4,AE4),0)</f>
         <v>8</v>
       </c>
@@ -6025,7 +6034,7 @@
         <f aca="false">ROUND(AVERAGE(C5,E5,J5),0)</f>
         <v>10</v>
       </c>
-      <c r="L5" s="8" t="str">
+      <c r="L5" s="9" t="str">
         <f aca="false">IF(K5&lt;7,"TEP","TEA")</f>
         <v>TEA</v>
       </c>
@@ -6035,7 +6044,7 @@
       <c r="N5" s="17" t="n">
         <v>45849</v>
       </c>
-      <c r="O5" s="7" t="n">
+      <c r="O5" s="8" t="n">
         <v>8</v>
       </c>
       <c r="P5" s="1" t="n">
@@ -6048,38 +6057,38 @@
       <c r="R5" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="S5" s="8" t="n">
+      <c r="S5" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(P5:R5),0)</f>
         <v>8</v>
       </c>
-      <c r="T5" s="8"/>
-      <c r="U5" s="8"/>
-      <c r="V5" s="8"/>
+      <c r="T5" s="9"/>
+      <c r="U5" s="9"/>
+      <c r="V5" s="9"/>
       <c r="Y5" s="1" t="n">
         <v>8</v>
       </c>
       <c r="Z5" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="AA5" s="0" t="n">
+      <c r="AA5" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="AC5" s="15" t="n">
+      <c r="AC5" s="1" t="n">
         <f aca="false">AA5+AB5/2</f>
         <v>7</v>
       </c>
-      <c r="AD5" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="AE5" s="15" t="n">
+      <c r="AD5" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="AE5" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(Y5,Z5,AC5),0)</f>
         <v>5</v>
       </c>
-      <c r="AF5" s="15" t="n">
+      <c r="AF5" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(AD5,AE5),0)</f>
         <v>7</v>
       </c>
-      <c r="AG5" s="15" t="n">
+      <c r="AG5" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(S5,AE5),0)</f>
         <v>7</v>
       </c>
@@ -6120,14 +6129,14 @@
         <f aca="false">ROUND(AVERAGE(C6,E6,J6),0)</f>
         <v>8</v>
       </c>
-      <c r="L6" s="8" t="str">
+      <c r="L6" s="9" t="str">
         <f aca="false">IF(K6&lt;7,"TEP","TEA")</f>
         <v>TEA</v>
       </c>
       <c r="M6" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="O6" s="7" t="n">
+      <c r="O6" s="8" t="n">
         <v>8</v>
       </c>
       <c r="P6" s="1" t="n">
@@ -6140,13 +6149,13 @@
       <c r="R6" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="S6" s="8" t="n">
+      <c r="S6" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(P6:R6),0)</f>
         <v>8</v>
       </c>
-      <c r="T6" s="8"/>
-      <c r="U6" s="8"/>
-      <c r="V6" s="8"/>
+      <c r="T6" s="9"/>
+      <c r="U6" s="9"/>
+      <c r="V6" s="9"/>
       <c r="W6" s="1" t="n">
         <v>7</v>
       </c>
@@ -6156,25 +6165,25 @@
       <c r="Z6" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="AA6" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC6" s="15" t="n">
+      <c r="AA6" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC6" s="1" t="n">
         <f aca="false">AA6+AB6/2</f>
         <v>10</v>
       </c>
-      <c r="AD6" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="AE6" s="15" t="n">
+      <c r="AD6" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE6" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(Y6,Z6,AC6),0)</f>
         <v>9</v>
       </c>
-      <c r="AF6" s="15" t="n">
+      <c r="AF6" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(AD6,AE6),0)</f>
         <v>10</v>
       </c>
-      <c r="AG6" s="15" t="n">
+      <c r="AG6" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(S6,AE6),0)</f>
         <v>9</v>
       </c>
@@ -6183,7 +6192,7 @@
       <c r="A7" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="11" t="s">
         <v>32</v>
       </c>
       <c r="C7" s="2" t="n">
@@ -6213,7 +6222,7 @@
       <c r="M7" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="O7" s="11" t="n">
+      <c r="O7" s="13" t="n">
         <v>1</v>
       </c>
       <c r="P7" s="2" t="n">
@@ -6242,23 +6251,23 @@
       <c r="AA7" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AB7" s="0"/>
-      <c r="AC7" s="0" t="n">
+      <c r="AB7" s="1"/>
+      <c r="AC7" s="1" t="n">
         <f aca="false">AA7+AB7/2</f>
         <v>1</v>
       </c>
-      <c r="AD7" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE7" s="15" t="n">
+      <c r="AD7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE7" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(Y7,Z7,AC7),0)</f>
         <v>3</v>
       </c>
-      <c r="AF7" s="15" t="n">
+      <c r="AF7" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(AD7,AE7),0)</f>
         <v>2</v>
       </c>
-      <c r="AG7" s="15" t="n">
+      <c r="AG7" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(S7,AE7),0)</f>
         <v>5</v>
       </c>
@@ -6267,7 +6276,7 @@
       <c r="A8" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="11" t="s">
         <v>35</v>
       </c>
       <c r="C8" s="2" t="n">
@@ -6297,7 +6306,7 @@
       <c r="M8" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="O8" s="11" t="n">
+      <c r="O8" s="13" t="n">
         <v>0</v>
       </c>
       <c r="P8" s="2" t="n">
@@ -6310,7 +6319,7 @@
       <c r="R8" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="S8" s="8" t="n">
+      <c r="S8" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(P8:R8),0)</f>
         <v>6</v>
       </c>
@@ -6332,23 +6341,23 @@
       <c r="AA8" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AB8" s="0"/>
-      <c r="AC8" s="0" t="n">
+      <c r="AB8" s="1"/>
+      <c r="AC8" s="1" t="n">
         <f aca="false">AA8+AB8/2</f>
         <v>1</v>
       </c>
-      <c r="AD8" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE8" s="15" t="n">
+      <c r="AD8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE8" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(Y8,Z8,AC8),0)</f>
         <v>1</v>
       </c>
-      <c r="AF8" s="15" t="n">
+      <c r="AF8" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(AD8,AE8),0)</f>
         <v>1</v>
       </c>
-      <c r="AG8" s="15" t="n">
+      <c r="AG8" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(S8,AE8),0)</f>
         <v>4</v>
       </c>
@@ -6383,14 +6392,14 @@
         <f aca="false">ROUND(AVERAGE(C9,E9,J9),0)</f>
         <v>8</v>
       </c>
-      <c r="L9" s="8" t="str">
+      <c r="L9" s="9" t="str">
         <f aca="false">IF(K9&lt;7,"TEP","TEA")</f>
         <v>TEA</v>
       </c>
       <c r="M9" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="O9" s="7" t="n">
+      <c r="O9" s="8" t="n">
         <v>10</v>
       </c>
       <c r="P9" s="1" t="n">
@@ -6403,7 +6412,7 @@
       <c r="R9" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="S9" s="8" t="n">
+      <c r="S9" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(P9:R9),0)</f>
         <v>8</v>
       </c>
@@ -6413,25 +6422,25 @@
       <c r="Z9" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="AA9" s="0" t="n">
+      <c r="AA9" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="AC9" s="15" t="n">
+      <c r="AC9" s="1" t="n">
         <f aca="false">AA9+AB9/2</f>
         <v>7</v>
       </c>
-      <c r="AD9" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="AE9" s="15" t="n">
+      <c r="AD9" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="AE9" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(Y9,Z9,AC9),0)</f>
         <v>8</v>
       </c>
-      <c r="AF9" s="15" t="n">
+      <c r="AF9" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(AD9,AE9),0)</f>
         <v>9</v>
       </c>
-      <c r="AG9" s="15" t="n">
+      <c r="AG9" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(S9,AE9),0)</f>
         <v>8</v>
       </c>
@@ -6469,14 +6478,14 @@
         <f aca="false">ROUND(AVERAGE(C10,E10,J10),0)</f>
         <v>9</v>
       </c>
-      <c r="L10" s="8" t="str">
+      <c r="L10" s="9" t="str">
         <f aca="false">IF(K10&lt;7,"TEP","TEA")</f>
         <v>TEA</v>
       </c>
       <c r="M10" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="O10" s="7" t="n">
+      <c r="O10" s="8" t="n">
         <v>10</v>
       </c>
       <c r="P10" s="1" t="n">
@@ -6489,7 +6498,7 @@
       <c r="R10" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="S10" s="8" t="n">
+      <c r="S10" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(P10:R10),0)</f>
         <v>9</v>
       </c>
@@ -6502,28 +6511,28 @@
       <c r="Z10" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="AA10" s="0" t="n">
+      <c r="AA10" s="1" t="n">
         <v>10</v>
       </c>
       <c r="AB10" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="AC10" s="15" t="n">
+      <c r="AC10" s="1" t="n">
         <f aca="false">AA10+AB10/2</f>
         <v>10.5</v>
       </c>
-      <c r="AD10" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="AE10" s="15" t="n">
+      <c r="AD10" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE10" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(Y10,Z10,AC10),0)</f>
         <v>10</v>
       </c>
-      <c r="AF10" s="15" t="n">
+      <c r="AF10" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(AD10,AE10),0)</f>
         <v>10</v>
       </c>
-      <c r="AG10" s="15" t="n">
+      <c r="AG10" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(S10,AE10),0)</f>
         <v>10</v>
       </c>
@@ -6555,14 +6564,14 @@
         <f aca="false">ROUND(AVERAGE(C11,E11,J11),0)</f>
         <v>11</v>
       </c>
-      <c r="L11" s="8" t="str">
+      <c r="L11" s="9" t="str">
         <f aca="false">IF(K11&lt;7,"TEP","TEA")</f>
         <v>TEA</v>
       </c>
       <c r="M11" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="O11" s="7" t="n">
+      <c r="O11" s="8" t="n">
         <v>10</v>
       </c>
       <c r="P11" s="1" t="n">
@@ -6575,7 +6584,7 @@
       <c r="R11" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="S11" s="8" t="n">
+      <c r="S11" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(P11:R11),0)</f>
         <v>9</v>
       </c>
@@ -6588,28 +6597,28 @@
       <c r="Z11" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="AA11" s="0" t="n">
+      <c r="AA11" s="1" t="n">
         <v>10</v>
       </c>
       <c r="AB11" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="AC11" s="15" t="n">
+      <c r="AC11" s="1" t="n">
         <f aca="false">AA11+AB11/2</f>
         <v>10.5</v>
       </c>
-      <c r="AD11" s="0" t="n">
-        <v>19</v>
-      </c>
-      <c r="AE11" s="15" t="n">
+      <c r="AD11" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="AE11" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(Y11,Z11,AC11),0)</f>
         <v>10</v>
       </c>
-      <c r="AF11" s="15" t="n">
+      <c r="AF11" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(AD11,AE11),0)</f>
         <v>15</v>
       </c>
-      <c r="AG11" s="15" t="n">
+      <c r="AG11" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(S11,AE11),0)</f>
         <v>10</v>
       </c>
@@ -6647,14 +6656,14 @@
         <f aca="false">ROUND(AVERAGE(C12,E12,J12),0)</f>
         <v>7</v>
       </c>
-      <c r="L12" s="8" t="str">
+      <c r="L12" s="9" t="str">
         <f aca="false">IF(K12&lt;7,"TEP","TEA")</f>
         <v>TEA</v>
       </c>
       <c r="M12" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="O12" s="7" t="n">
+      <c r="O12" s="8" t="n">
         <v>9</v>
       </c>
       <c r="P12" s="1" t="n">
@@ -6667,7 +6676,7 @@
       <c r="R12" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="S12" s="8" t="n">
+      <c r="S12" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(P12:R12),0)</f>
         <v>7</v>
       </c>
@@ -6677,28 +6686,28 @@
       <c r="Z12" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="AA12" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB12" s="14" t="n">
+      <c r="AA12" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB12" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="AC12" s="15" t="n">
+      <c r="AC12" s="1" t="n">
         <f aca="false">AA12+AB12/2</f>
         <v>3.5</v>
       </c>
-      <c r="AD12" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="AE12" s="15" t="n">
+      <c r="AD12" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="AE12" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(Y12,Z12,AC12),0)</f>
         <v>7</v>
       </c>
-      <c r="AF12" s="15" t="n">
+      <c r="AF12" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(AD12,AE12),0)</f>
         <v>8</v>
       </c>
-      <c r="AG12" s="15" t="n">
+      <c r="AG12" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(S12,AE12),0)</f>
         <v>7</v>
       </c>
@@ -6730,14 +6739,14 @@
         <f aca="false">ROUND(AVERAGE(C13,E13,J13),0)</f>
         <v>5</v>
       </c>
-      <c r="L13" s="8" t="str">
+      <c r="L13" s="9" t="str">
         <f aca="false">IF(K13&lt;7,"TEP","TEA")</f>
         <v>TEP</v>
       </c>
       <c r="M13" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="O13" s="7" t="n">
+      <c r="O13" s="8" t="n">
         <v>10</v>
       </c>
       <c r="P13" s="1" t="n">
@@ -6750,7 +6759,7 @@
       <c r="R13" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="S13" s="8" t="n">
+      <c r="S13" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(P13:R13),0)</f>
         <v>8</v>
       </c>
@@ -6760,25 +6769,25 @@
       <c r="Z13" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="AA13" s="0" t="n">
+      <c r="AA13" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="AC13" s="15" t="n">
+      <c r="AC13" s="1" t="n">
         <f aca="false">AA13+AB13/2</f>
         <v>7</v>
       </c>
-      <c r="AD13" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="AE13" s="15" t="n">
+      <c r="AD13" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="AE13" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(Y13,Z13,AC13),0)</f>
         <v>8</v>
       </c>
-      <c r="AF13" s="15" t="n">
+      <c r="AF13" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(AD13,AE13),0)</f>
         <v>9</v>
       </c>
-      <c r="AG13" s="15" t="n">
+      <c r="AG13" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(S13,AE13),0)</f>
         <v>8</v>
       </c>
@@ -6819,14 +6828,14 @@
         <f aca="false">ROUND(AVERAGE(C14,E14,J14),0)</f>
         <v>8</v>
       </c>
-      <c r="L14" s="8" t="str">
+      <c r="L14" s="9" t="str">
         <f aca="false">IF(K14&lt;7,"TEP","TEA")</f>
         <v>TEA</v>
       </c>
       <c r="M14" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="O14" s="7" t="n">
+      <c r="O14" s="8" t="n">
         <v>8</v>
       </c>
       <c r="P14" s="1" t="n">
@@ -6839,7 +6848,7 @@
       <c r="R14" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="S14" s="8" t="n">
+      <c r="S14" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(P14:R14),0)</f>
         <v>8</v>
       </c>
@@ -6852,25 +6861,25 @@
       <c r="Z14" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="AA14" s="0" t="n">
-        <v>8</v>
-      </c>
-      <c r="AC14" s="15" t="n">
+      <c r="AA14" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="AC14" s="1" t="n">
         <f aca="false">AA14+AB14/2</f>
         <v>8</v>
       </c>
-      <c r="AD14" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="AE14" s="15" t="n">
+      <c r="AD14" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE14" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(Y14,Z14,AC14),0)</f>
         <v>9</v>
       </c>
-      <c r="AF14" s="15" t="n">
+      <c r="AF14" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(AD14,AE14),0)</f>
         <v>10</v>
       </c>
-      <c r="AG14" s="15" t="n">
+      <c r="AG14" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(S14,AE14),0)</f>
         <v>9</v>
       </c>
@@ -6902,14 +6911,14 @@
         <f aca="false">ROUND(AVERAGE(C15,E15,J15),0)</f>
         <v>11</v>
       </c>
-      <c r="L15" s="8" t="str">
+      <c r="L15" s="9" t="str">
         <f aca="false">IF(K15&lt;7,"TEP","TEA")</f>
         <v>TEA</v>
       </c>
       <c r="M15" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="O15" s="7" t="n">
+      <c r="O15" s="8" t="n">
         <v>7</v>
       </c>
       <c r="P15" s="1" t="n">
@@ -6922,7 +6931,7 @@
       <c r="R15" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="S15" s="8" t="n">
+      <c r="S15" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(P15:R15),0)</f>
         <v>9</v>
       </c>
@@ -6932,25 +6941,25 @@
       <c r="Z15" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="AA15" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC15" s="15" t="n">
+      <c r="AA15" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC15" s="1" t="n">
         <f aca="false">AA15+AB15/2</f>
         <v>10</v>
       </c>
-      <c r="AD15" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="AE15" s="15" t="n">
+      <c r="AD15" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="AE15" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(Y15,Z15,AC15),0)</f>
         <v>10</v>
       </c>
-      <c r="AF15" s="15" t="n">
+      <c r="AF15" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(AD15,AE15),0)</f>
         <v>10</v>
       </c>
-      <c r="AG15" s="15" t="n">
+      <c r="AG15" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(S15,AE15),0)</f>
         <v>10</v>
       </c>
@@ -6981,14 +6990,14 @@
         <f aca="false">ROUND(AVERAGE(C16,E16,J16),0)</f>
         <v>15</v>
       </c>
-      <c r="L16" s="8" t="str">
+      <c r="L16" s="9" t="str">
         <f aca="false">IF(K16&lt;7,"TEP","TEA")</f>
         <v>TEA</v>
       </c>
       <c r="M16" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="O16" s="7" t="n">
+      <c r="O16" s="8" t="n">
         <v>8</v>
       </c>
       <c r="P16" s="1" t="n">
@@ -7001,7 +7010,7 @@
       <c r="R16" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="S16" s="8" t="n">
+      <c r="S16" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(P16:R16),0)</f>
         <v>8</v>
       </c>
@@ -7011,25 +7020,25 @@
       <c r="Z16" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="AA16" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC16" s="15" t="n">
+      <c r="AA16" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC16" s="1" t="n">
         <f aca="false">AA16+AB16/2</f>
         <v>10</v>
       </c>
-      <c r="AD16" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="AE16" s="15" t="n">
+      <c r="AD16" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="AE16" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(Y16,Z16,AC16),0)</f>
         <v>8</v>
       </c>
-      <c r="AF16" s="15" t="n">
+      <c r="AF16" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(AD16,AE16),0)</f>
         <v>9</v>
       </c>
-      <c r="AG16" s="15" t="n">
+      <c r="AG16" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(S16,AE16),0)</f>
         <v>8</v>
       </c>
@@ -7038,7 +7047,7 @@
       <c r="A17" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C17" s="2" t="n">
@@ -7074,7 +7083,7 @@
       <c r="N17" s="17" t="n">
         <v>45881</v>
       </c>
-      <c r="O17" s="11" t="n">
+      <c r="O17" s="13" t="n">
         <v>2</v>
       </c>
       <c r="P17" s="2" t="n">
@@ -7087,7 +7096,7 @@
       <c r="R17" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="S17" s="8" t="n">
+      <c r="S17" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(P17:R17),0)</f>
         <v>7</v>
       </c>
@@ -7106,23 +7115,23 @@
       <c r="Z17" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AB17" s="0"/>
-      <c r="AC17" s="0" t="n">
+      <c r="AB17" s="1"/>
+      <c r="AC17" s="1" t="n">
         <f aca="false">AA17+AB17/2</f>
         <v>0</v>
       </c>
-      <c r="AD17" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE17" s="15" t="n">
+      <c r="AD17" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE17" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(Y17,Z17,AC17),0)</f>
         <v>1</v>
       </c>
-      <c r="AF17" s="15" t="n">
+      <c r="AF17" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(AD17,AE17),0)</f>
         <v>1</v>
       </c>
-      <c r="AG17" s="15" t="n">
+      <c r="AG17" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(S17,AE17),0)</f>
         <v>4</v>
       </c>
@@ -7131,7 +7140,7 @@
       <c r="A18" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="B18" s="11" t="s">
         <v>68</v>
       </c>
       <c r="C18" s="2" t="n">
@@ -7167,7 +7176,7 @@
       <c r="M18" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="O18" s="11" t="n">
+      <c r="O18" s="13" t="n">
         <v>2</v>
       </c>
       <c r="P18" s="2" t="n">
@@ -7180,7 +7189,7 @@
       <c r="R18" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="S18" s="8" t="n">
+      <c r="S18" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(P18:R18),0)</f>
         <v>7</v>
       </c>
@@ -7203,23 +7212,23 @@
       <c r="AA18" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AB18" s="0"/>
-      <c r="AC18" s="0" t="n">
+      <c r="AB18" s="1"/>
+      <c r="AC18" s="1" t="n">
         <f aca="false">AA18+AB18/2</f>
         <v>1</v>
       </c>
-      <c r="AD18" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE18" s="15" t="n">
+      <c r="AD18" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE18" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(Y18,Z18,AC18),0)</f>
         <v>2</v>
       </c>
-      <c r="AF18" s="15" t="n">
+      <c r="AF18" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(AD18,AE18),0)</f>
         <v>2</v>
       </c>
-      <c r="AG18" s="15" t="n">
+      <c r="AG18" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(S18,AE18),0)</f>
         <v>5</v>
       </c>
@@ -7254,14 +7263,14 @@
         <f aca="false">ROUND(AVERAGE(C19,E19,J19),0)</f>
         <v>8</v>
       </c>
-      <c r="L19" s="8" t="str">
+      <c r="L19" s="9" t="str">
         <f aca="false">IF(K19&lt;7,"TEP","TEA")</f>
         <v>TEA</v>
       </c>
       <c r="M19" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="O19" s="7" t="n">
+      <c r="O19" s="8" t="n">
         <v>9</v>
       </c>
       <c r="P19" s="1" t="n">
@@ -7274,7 +7283,7 @@
       <c r="R19" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="S19" s="8" t="n">
+      <c r="S19" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(P19:R19),0)</f>
         <v>8</v>
       </c>
@@ -7284,25 +7293,25 @@
       <c r="Z19" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="AA19" s="0" t="n">
-        <v>8</v>
-      </c>
-      <c r="AC19" s="15" t="n">
+      <c r="AA19" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="AC19" s="1" t="n">
         <f aca="false">AA19+AB19/2</f>
         <v>8</v>
       </c>
-      <c r="AD19" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="AE19" s="15" t="n">
+      <c r="AD19" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="AE19" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(Y19,Z19,AC19),0)</f>
         <v>9</v>
       </c>
-      <c r="AF19" s="15" t="n">
+      <c r="AF19" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(AD19,AE19),0)</f>
         <v>9</v>
       </c>
-      <c r="AG19" s="15" t="n">
+      <c r="AG19" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(S19,AE19),0)</f>
         <v>9</v>
       </c>
@@ -7334,14 +7343,14 @@
         <f aca="false">ROUND(AVERAGE(C20,E20,J20),0)</f>
         <v>7</v>
       </c>
-      <c r="L20" s="8" t="str">
+      <c r="L20" s="9" t="str">
         <f aca="false">IF(K20&lt;7,"TEP","TEA")</f>
         <v>TEA</v>
       </c>
       <c r="M20" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="O20" s="7" t="n">
+      <c r="O20" s="8" t="n">
         <v>9</v>
       </c>
       <c r="P20" s="1" t="n">
@@ -7354,7 +7363,7 @@
       <c r="R20" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="S20" s="8" t="n">
+      <c r="S20" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(P20:R20),0)</f>
         <v>8</v>
       </c>
@@ -7367,28 +7376,28 @@
       <c r="Z20" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="AA20" s="0" t="n">
+      <c r="AA20" s="1" t="n">
         <v>8</v>
       </c>
       <c r="AB20" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="AC20" s="15" t="n">
+      <c r="AC20" s="1" t="n">
         <f aca="false">AA20+AB20/2</f>
         <v>8.5</v>
       </c>
-      <c r="AD20" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="AE20" s="15" t="n">
+      <c r="AD20" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE20" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(Y20,Z20,AC20),0)</f>
         <v>8</v>
       </c>
-      <c r="AF20" s="15" t="n">
+      <c r="AF20" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(AD20,AE20),0)</f>
         <v>9</v>
       </c>
-      <c r="AG20" s="15" t="n">
+      <c r="AG20" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(S20,AE20),0)</f>
         <v>8</v>
       </c>
@@ -7423,14 +7432,14 @@
         <f aca="false">ROUND(AVERAGE(C21,E21,J21),0)</f>
         <v>10</v>
       </c>
-      <c r="L21" s="8" t="str">
+      <c r="L21" s="9" t="str">
         <f aca="false">IF(K21&lt;7,"TEP","TEA")</f>
         <v>TEA</v>
       </c>
       <c r="M21" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="O21" s="7" t="n">
+      <c r="O21" s="8" t="n">
         <v>10</v>
       </c>
       <c r="P21" s="1" t="n">
@@ -7443,7 +7452,7 @@
       <c r="R21" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="S21" s="8" t="n">
+      <c r="S21" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(P21:R21),0)</f>
         <v>9</v>
       </c>
@@ -7453,28 +7462,28 @@
       <c r="Z21" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="AA21" s="0" t="n">
+      <c r="AA21" s="1" t="n">
         <v>8</v>
       </c>
       <c r="AB21" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="AC21" s="15" t="n">
+      <c r="AC21" s="1" t="n">
         <f aca="false">AA21+AB21/2</f>
         <v>8.5</v>
       </c>
-      <c r="AD21" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="AE21" s="15" t="n">
+      <c r="AD21" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="AE21" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(Y21,Z21,AC21),0)</f>
         <v>7</v>
       </c>
-      <c r="AF21" s="15" t="n">
+      <c r="AF21" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(AD21,AE21),0)</f>
         <v>8</v>
       </c>
-      <c r="AG21" s="15" t="n">
+      <c r="AG21" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(S21,AE21),0)</f>
         <v>8</v>
       </c>
@@ -7506,14 +7515,14 @@
         <f aca="false">ROUND(AVERAGE(C22,E22,J22),0)</f>
         <v>1</v>
       </c>
-      <c r="L22" s="8" t="str">
+      <c r="L22" s="9" t="str">
         <f aca="false">IF(K22&lt;7,"TEP","TEA")</f>
         <v>TEP</v>
       </c>
       <c r="M22" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="O22" s="7" t="n">
+      <c r="O22" s="8" t="n">
         <v>1</v>
       </c>
       <c r="P22" s="1" t="n">
@@ -7526,7 +7535,7 @@
       <c r="R22" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="S22" s="8" t="n">
+      <c r="S22" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(P22:R22),0)</f>
         <v>6</v>
       </c>
@@ -7539,25 +7548,25 @@
       <c r="Z22" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="AA22" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC22" s="15" t="n">
+      <c r="AA22" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC22" s="1" t="n">
         <f aca="false">AA22+AB22/2</f>
         <v>1</v>
       </c>
-      <c r="AD22" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE22" s="15" t="n">
+      <c r="AD22" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE22" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(Y22,Z22,AC22),0)</f>
         <v>1</v>
       </c>
-      <c r="AF22" s="15" t="n">
+      <c r="AF22" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(AD22,AE22),0)</f>
         <v>1</v>
       </c>
-      <c r="AG22" s="15" t="n">
+      <c r="AG22" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(S22,AE22),0)</f>
         <v>4</v>
       </c>
@@ -7589,14 +7598,14 @@
         <f aca="false">ROUND(AVERAGE(C23,E23,J23),0)</f>
         <v>10</v>
       </c>
-      <c r="L23" s="8" t="str">
+      <c r="L23" s="9" t="str">
         <f aca="false">IF(K23&lt;7,"TEP","TEA")</f>
         <v>TEA</v>
       </c>
       <c r="M23" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="O23" s="7" t="n">
+      <c r="O23" s="8" t="n">
         <v>10</v>
       </c>
       <c r="P23" s="1" t="n">
@@ -7609,7 +7618,7 @@
       <c r="R23" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="S23" s="8" t="n">
+      <c r="S23" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(P23:R23),0)</f>
         <v>8</v>
       </c>
@@ -7619,25 +7628,25 @@
       <c r="Z23" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="AA23" s="0" t="n">
+      <c r="AA23" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="AC23" s="15" t="n">
+      <c r="AC23" s="1" t="n">
         <f aca="false">AA23+AB23/2</f>
         <v>7</v>
       </c>
-      <c r="AD23" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="AE23" s="15" t="n">
+      <c r="AD23" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="AE23" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(Y23,Z23,AC23),0)</f>
         <v>8</v>
       </c>
-      <c r="AF23" s="15" t="n">
+      <c r="AF23" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(AD23,AE23),0)</f>
         <v>9</v>
       </c>
-      <c r="AG23" s="15" t="n">
+      <c r="AG23" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(S23,AE23),0)</f>
         <v>8</v>
       </c>
@@ -7670,14 +7679,14 @@
         <f aca="false">ROUND(AVERAGE(C24,E24,J24),0)</f>
         <v>12</v>
       </c>
-      <c r="L24" s="8" t="str">
+      <c r="L24" s="9" t="str">
         <f aca="false">IF(K24&lt;7,"TEP","TEA")</f>
         <v>TEA</v>
       </c>
       <c r="M24" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="O24" s="7" t="n">
+      <c r="O24" s="8" t="n">
         <v>8</v>
       </c>
       <c r="P24" s="1" t="n">
@@ -7690,7 +7699,7 @@
       <c r="R24" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="S24" s="8" t="n">
+      <c r="S24" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(P24:R24),0)</f>
         <v>9</v>
       </c>
@@ -7700,28 +7709,28 @@
       <c r="Z24" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="AA24" s="0" t="n">
+      <c r="AA24" s="1" t="n">
         <v>10</v>
       </c>
       <c r="AB24" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="AC24" s="15" t="n">
+      <c r="AC24" s="1" t="n">
         <f aca="false">AA24+AB24/2</f>
         <v>10.5</v>
       </c>
-      <c r="AD24" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="AE24" s="15" t="n">
+      <c r="AD24" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE24" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(Y24,Z24,AC24),0)</f>
         <v>10</v>
       </c>
-      <c r="AF24" s="15" t="n">
+      <c r="AF24" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(AD24,AE24),0)</f>
         <v>10</v>
       </c>
-      <c r="AG24" s="15" t="n">
+      <c r="AG24" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(S24,AE24),0)</f>
         <v>10</v>
       </c>
@@ -7753,14 +7762,14 @@
         <f aca="false">ROUND(AVERAGE(C25,E25,J25),0)</f>
         <v>12</v>
       </c>
-      <c r="L25" s="8" t="str">
+      <c r="L25" s="9" t="str">
         <f aca="false">IF(K25&lt;7,"TEP","TEA")</f>
         <v>TEA</v>
       </c>
       <c r="M25" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="O25" s="7" t="n">
+      <c r="O25" s="8" t="n">
         <v>9</v>
       </c>
       <c r="P25" s="1" t="n">
@@ -7773,7 +7782,7 @@
       <c r="R25" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="S25" s="8" t="n">
+      <c r="S25" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(P25:R25),0)</f>
         <v>9</v>
       </c>
@@ -7786,25 +7795,25 @@
       <c r="Z25" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="AA25" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC25" s="15" t="n">
+      <c r="AA25" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC25" s="1" t="n">
         <f aca="false">AA25+AB25/2</f>
         <v>10</v>
       </c>
-      <c r="AD25" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="AE25" s="15" t="n">
+      <c r="AD25" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="AE25" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(Y25,Z25,AC25),0)</f>
         <v>10</v>
       </c>
-      <c r="AF25" s="15" t="n">
+      <c r="AF25" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(AD25,AE25),0)</f>
         <v>10</v>
       </c>
-      <c r="AG25" s="15" t="n">
+      <c r="AG25" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(S25,AE25),0)</f>
         <v>10</v>
       </c>
@@ -7836,14 +7845,14 @@
         <f aca="false">ROUND(AVERAGE(C26,E26,J26),0)</f>
         <v>15</v>
       </c>
-      <c r="L26" s="8" t="str">
+      <c r="L26" s="9" t="str">
         <f aca="false">IF(K26&lt;7,"TEP","TEA")</f>
         <v>TEA</v>
       </c>
       <c r="M26" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="O26" s="7" t="n">
+      <c r="O26" s="8" t="n">
         <v>9</v>
       </c>
       <c r="P26" s="1" t="n">
@@ -7856,7 +7865,7 @@
       <c r="R26" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="S26" s="8" t="n">
+      <c r="S26" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(P26:R26),0)</f>
         <v>10</v>
       </c>
@@ -7866,25 +7875,25 @@
       <c r="Z26" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="AA26" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC26" s="15" t="n">
+      <c r="AA26" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC26" s="1" t="n">
         <f aca="false">AA26+AB26/2</f>
         <v>10</v>
       </c>
-      <c r="AD26" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="AE26" s="15" t="n">
+      <c r="AD26" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="AE26" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(Y26,Z26,AC26),0)</f>
         <v>10</v>
       </c>
-      <c r="AF26" s="15" t="n">
+      <c r="AF26" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(AD26,AE26),0)</f>
         <v>10</v>
       </c>
-      <c r="AG26" s="15" t="n">
+      <c r="AG26" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(S26,AE26),0)</f>
         <v>10</v>
       </c>
@@ -7916,14 +7925,14 @@
         <f aca="false">ROUND(AVERAGE(C27,E27,J27),0)</f>
         <v>14</v>
       </c>
-      <c r="L27" s="8" t="str">
+      <c r="L27" s="9" t="str">
         <f aca="false">IF(K27&lt;7,"TEP","TEA")</f>
         <v>TEA</v>
       </c>
       <c r="M27" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="O27" s="7" t="n">
+      <c r="O27" s="8" t="n">
         <v>10</v>
       </c>
       <c r="P27" s="1" t="n">
@@ -7936,7 +7945,7 @@
       <c r="R27" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="S27" s="8" t="n">
+      <c r="S27" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(P27:R27),0)</f>
         <v>9</v>
       </c>
@@ -7946,28 +7955,28 @@
       <c r="Z27" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="AA27" s="0" t="n">
+      <c r="AA27" s="1" t="n">
         <v>8</v>
       </c>
       <c r="AB27" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="AC27" s="15" t="n">
+      <c r="AC27" s="1" t="n">
         <f aca="false">AA27+AB27/2</f>
         <v>8.5</v>
       </c>
-      <c r="AD27" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="AE27" s="15" t="n">
+      <c r="AD27" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE27" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(Y27,Z27,AC27),0)</f>
         <v>9</v>
       </c>
-      <c r="AF27" s="15" t="n">
+      <c r="AF27" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(AD27,AE27),0)</f>
         <v>10</v>
       </c>
-      <c r="AG27" s="15" t="n">
+      <c r="AG27" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(S27,AE27),0)</f>
         <v>9</v>
       </c>
@@ -7976,7 +7985,7 @@
       <c r="A28" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="B28" s="9" t="s">
+      <c r="B28" s="11" t="s">
         <v>99</v>
       </c>
       <c r="C28" s="2" t="n">
@@ -8006,7 +8015,7 @@
       <c r="M28" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="O28" s="11" t="n">
+      <c r="O28" s="13" t="n">
         <v>0</v>
       </c>
       <c r="P28" s="2" t="n">
@@ -8019,7 +8028,7 @@
       <c r="R28" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="S28" s="8" t="n">
+      <c r="S28" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(P28:R28),0)</f>
         <v>6</v>
       </c>
@@ -8041,22 +8050,22 @@
       <c r="AA28" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AC28" s="15" t="n">
+      <c r="AC28" s="1" t="n">
         <f aca="false">AA28+AB28/2</f>
         <v>1</v>
       </c>
-      <c r="AD28" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE28" s="15" t="n">
+      <c r="AD28" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE28" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(Y28,Z28,AC28),0)</f>
         <v>1</v>
       </c>
-      <c r="AF28" s="15" t="n">
+      <c r="AF28" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(AD28,AE28),0)</f>
         <v>1</v>
       </c>
-      <c r="AG28" s="15" t="n">
+      <c r="AG28" s="9" t="n">
         <f aca="false">ROUND(AVERAGE(S28,AE28),0)</f>
         <v>4</v>
       </c>

</xml_diff>